<commit_message>
Añadida cobertura QQQ configurable
</commit_message>
<xml_diff>
--- a/USAstocks.xlsx
+++ b/USAstocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TE237142\iCloudDrive\Docs Arnau\Forex\Fx2020\EvolucioInvertim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29B6620-31BB-426D-B9E4-9FAC9331BB69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2867BB72-4C71-4103-8946-51BECBA84B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
   <si>
     <t>Ticker</t>
   </si>
@@ -211,6 +211,12 @@
   </si>
   <si>
     <t>ECHO</t>
+  </si>
+  <si>
+    <t>QQQ</t>
+  </si>
+  <si>
+    <t>Invesco QQQ Trust</t>
   </si>
 </sst>
 </file>
@@ -558,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
@@ -906,6 +912,17 @@
         <v>46235</v>
       </c>
     </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="3">
+        <v>46196</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Restaurar dashboard anterior sin cobertura
</commit_message>
<xml_diff>
--- a/USAstocks.xlsx
+++ b/USAstocks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TE237142\iCloudDrive\Docs Arnau\Forex\Fx2020\EvolucioInvertim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2867BB72-4C71-4103-8946-51BECBA84B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA5A469A-5D51-4004-853A-FE588AD26D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
   <si>
     <t>Ticker</t>
   </si>
@@ -211,12 +211,6 @@
   </si>
   <si>
     <t>ECHO</t>
-  </si>
-  <si>
-    <t>QQQ</t>
-  </si>
-  <si>
-    <t>Invesco QQQ Trust</t>
   </si>
 </sst>
 </file>
@@ -564,19 +558,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,7 +590,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -613,7 +607,7 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -630,7 +624,7 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -647,7 +641,7 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -667,7 +661,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -687,7 +681,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -707,7 +701,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -727,7 +721,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -747,7 +741,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -764,7 +758,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -784,7 +778,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -804,7 +798,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -821,7 +815,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -838,7 +832,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>61</v>
       </c>
@@ -858,7 +852,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -878,7 +872,7 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -895,7 +889,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -910,17 +904,6 @@
       </c>
       <c r="E18" s="3">
         <v>46235</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="3">
-        <v>46196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadidas coberturas multiples QQQ
</commit_message>
<xml_diff>
--- a/USAstocks.xlsx
+++ b/USAstocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TE237142\iCloudDrive\Docs Arnau\Forex\Fx2020\EvolucioInvertim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA5A469A-5D51-4004-853A-FE588AD26D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8AB418-8F73-41C8-8AD8-73DD3378B690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="64">
   <si>
     <t>Ticker</t>
   </si>
@@ -211,6 +211,12 @@
   </si>
   <si>
     <t>ECHO</t>
+  </si>
+  <si>
+    <t>QQQ</t>
+  </si>
+  <si>
+    <t>Invesco QQQ Trust</t>
   </si>
 </sst>
 </file>
@@ -558,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
@@ -906,6 +912,102 @@
         <v>46235</v>
       </c>
     </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="3">
+        <v>46048</v>
+      </c>
+      <c r="D21" s="3">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="3">
+        <v>46104</v>
+      </c>
+      <c r="D22" s="3">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="3">
+        <v>46139</v>
+      </c>
+      <c r="D23" s="3">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="3">
+        <v>46153</v>
+      </c>
+      <c r="D24" s="3">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="3">
+        <v>46181</v>
+      </c>
+      <c r="D25" s="3">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="3">
+        <v>46195</v>
+      </c>
+      <c r="D26" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
añado MRNA y saco CIEN
</commit_message>
<xml_diff>
--- a/USAstocks.xlsx
+++ b/USAstocks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TE237142\iCloudDrive\Docs Arnau\Forex\Fx2020\EvolucioInvertim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8AB418-8F73-41C8-8AD8-73DD3378B690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD13CFCA-B5D3-47F6-8082-4CB3825A16FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-1230" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
   <si>
     <t>Ticker</t>
   </si>
@@ -217,6 +217,18 @@
   </si>
   <si>
     <t>Invesco QQQ Trust</t>
+  </si>
+  <si>
+    <t>MRNA</t>
+  </si>
+  <si>
+    <t>Moderna Inc</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Medical - Biomedical</t>
   </si>
 </sst>
 </file>
@@ -564,19 +576,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.7265625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -596,7 +608,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -613,7 +625,7 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -630,7 +642,7 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -647,7 +659,7 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -667,7 +679,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -687,7 +699,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -707,7 +719,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -727,7 +739,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -747,7 +759,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -764,7 +776,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -784,7 +796,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -804,7 +816,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -821,7 +833,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -837,8 +849,11 @@
       <c r="E14" s="3">
         <v>46113</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F14" s="3">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>61</v>
       </c>
@@ -858,7 +873,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -878,7 +893,7 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -895,7 +910,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -912,35 +927,38 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="3">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="3">
-        <v>46048</v>
-      </c>
-      <c r="D21" s="3">
-        <v>46097</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>62</v>
       </c>
@@ -948,13 +966,13 @@
         <v>63</v>
       </c>
       <c r="C22" s="3">
-        <v>46104</v>
+        <v>46048</v>
       </c>
       <c r="D22" s="3">
-        <v>46111</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -962,13 +980,13 @@
         <v>63</v>
       </c>
       <c r="C23" s="3">
-        <v>46139</v>
+        <v>46104</v>
       </c>
       <c r="D23" s="3">
-        <v>46146</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -976,13 +994,13 @@
         <v>63</v>
       </c>
       <c r="C24" s="3">
-        <v>46153</v>
+        <v>46139</v>
       </c>
       <c r="D24" s="3">
-        <v>46174</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -990,13 +1008,13 @@
         <v>63</v>
       </c>
       <c r="C25" s="3">
-        <v>46181</v>
+        <v>46153</v>
       </c>
       <c r="D25" s="3">
-        <v>46188</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>62</v>
       </c>
@@ -1004,9 +1022,23 @@
         <v>63</v>
       </c>
       <c r="C26" s="3">
+        <v>46181</v>
+      </c>
+      <c r="D26" s="3">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="3">
         <v>46195</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D27" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>